<commit_message>
Feature workbook: whole careers retired (iteration 83); the 968's verify and parity in the debut market block's evidence
1,372 features, 2,945 formulas, recalculated with no errors.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016u1Fo7XhbdeBDHcXP4s8th
</commit_message>
<xml_diff>
--- a/reports/feature_inventory.xlsx
+++ b/reports/feature_inventory.xlsx
@@ -8956,7 +8956,7 @@
     <t xml:space="preserve">Iteration 73 (steadier screen, on the 853): beside form lines and connection windows +0.0017 (+0.0003 to +0.0033), resolved worse, the outsiders +0.0074: the third pedigree reading to fail. Retired.</t>
   </si>
   <si>
-    <t xml:space="preserve">Iteration 75 (screen): -0.0011, unresolved; maiden, novice and bumper races -0.0048. Iteration 80 (served recipe, Huber): -0.0032 beside the 958h, those races -0.0067. Iteration 81 (served recipe, squared error): -0.0018 (-0.0028 to -0.0008) beside the 958, concordance resolved better. In the 968, the next candidate (train-bfsp run 41; its Huber twin run 42).</t>
+    <t xml:space="preserve">Iteration 75 (screen): -0.0011, unresolved; maiden, novice and bumper races -0.0048. Iteration 80 (served recipe, Huber): -0.0032 beside the 958h, those races -0.0067. Iteration 81 (served recipe, squared error): -0.0018 (-0.0028 to -0.0008) beside the 958, concordance resolved better. In the 968, the next candidate (train-bfsp run 41: verify PASS, parity clean, every feature identical on the 06:00 card; its Huber twin run 42).</t>
   </si>
   <si>
     <t xml:space="preserve">Iteration 69 (steadier screen, on the 853): -0.0056 (-0.0072 to -0.0041) alone, but beside form lines and connection windows -0.0008 (-0.0021 to +0.0005), unresolved, the early-price rule +7.84% against +8.47%: what it reads, connection windows already carry. Retired.</t>
@@ -8971,7 +8971,7 @@
     <t xml:space="preserve">Built 26 Sep beside the debut market block: the engine reads the pedigree only by results. Iteration 84 (the 968 + the block, two seeds each, served recipe) queued.</t>
   </si>
   <si>
-    <t xml:space="preserve">Built 26 Sep from a table of every horse's runs before 2021 (114,078 horses, 1.31m runs): 74% of 2021's runs, 47% of 2022's and 8% of the development window's have such a record. Iteration 83 (the 958 + the block, served recipe) under test.</t>
+    <t xml:space="preserve">Built 26 Sep from a table of every horse's runs before 2021 (114,078 horses, 1.31m runs): 74% of 2021's runs, 47% of 2022's and 8% of the development window's have such a record. Iteration 83 (the 958 + the block, served recipe): against four refits of the 958 -0.0008 to +0.0002; on the 4,330 runners with a pre-2021 record +0.0010. Retired.</t>
   </si>
   <si>
     <t xml:space="preserve">Iteration 35: -0.0004; iteration 54 (steadier screen): -0.0009 (-0.0023 to +0.0003): nothing.</t>

</xml_diff>

<commit_message>
Feature workbook: the not-yet-developed list takes the 27 Sep screen's readings
Weight per OR point leaves the list: the handicap angles' hca_wt_vs_mark is it, the fourth feature
by gain in run 52. Weight against the last three runs joins it as the next small candidate (the
screen read -2.14 x 10^-4, resolved; the model reads weight against the last run only). Lengths
per place, the headgear items, the rating's slope and peak, the OR percentile and the class ladder
carry what the screen found for them (misc_residuals: nothing, or unresolved) and stay low. No
formula errors (3,168 formulas).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016u1Fo7XhbdeBDHcXP4s8th
</commit_message>
<xml_diff>
--- a/reports/feature_inventory.xlsx
+++ b/reports/feature_inventory.xlsx
@@ -71,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10784" uniqueCount="3358">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10784" uniqueCount="3359">
   <si>
     <t xml:space="preserve">Ashcroft price model: feature inventory</t>
   </si>
@@ -9811,187 +9811,190 @@
     <t xml:space="preserve">Lengths beaten per place behind the winner (how strung out the field was)</t>
   </si>
   <si>
+    <t xml:space="preserve">Screened (research query misc_residuals, 27 Sep, x 10^-4 on the pair's mean |log error|): the last race's lengths per place and the horse's lengths against it +0.66 jointly, nothing. Not built</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Closing-sectional proxy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Speed over the final furlongs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not available</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No sectional or per-horse times in the data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Headgear type flags</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equipment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One flag per headgear item (blinkers, visor, cheekpieces, hood, tongue-tie)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partial: one category column. Screened (research query misc_residuals, 27 Sep, x 10^-4 on the pair's mean |log error|): each item worn, the number worn and headgear taken off -0.98 jointly (-2.23 to +0.24), unresolved; the items alone -0.76, resolved</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Age restriction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Race conditions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Age band of the race (2yo, 3yo only, 3yo+, 4yo+)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">race_restrictions_age is never read</t>
+  </si>
+  <si>
+    <t xml:space="preserve">H3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Claimer flag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Connections</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Whether the jockey claims an allowance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partial: raw claim only; is_claimer is opt-in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OR percentile in the field</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ratings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Official rating's percentile within the race</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partial: difference to the max and median only. Screened (research query misc_residuals, 27 Sep, x 10^-4 on the pair's mean |log error|) with the rating ladder: nothing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OR trajectory slope</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slope of the official rating over recent runs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partial: changes only. Screened (research query misc_residuals, 27 Sep, x 10^-4 on the pair's mean |log error|): the rating's slope over three runs and against its peak, with the class ladder, -0.85 jointly (-2.33 to +0.55), unresolved; against the peak alone -0.72</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Month / season</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Context</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seasonal effects</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Surveyed on 24 Sep: nothing for the price to miss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Day of week</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weekday effects (strength of meetings)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Surveyed: nothing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campaign stage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run number within the current campaign</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Written in model/primitives.py, never called; fr_runs_since_break now covers most of it</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Major-race experience</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Class</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Runs and form in Group / Listed / major races</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Screened 27 Sep against the best model's errors (black-type runs, finishing position and win rate before today: +0.53 x 10^-4, nothing; research/queries/travel_residuals.py)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Class ladder vs career median</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Today's class against the horse's career median class</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partial: against a three-run mean. Screened (research query misc_residuals, 27 Sep, x 10^-4 on the pair's mean |log error|) against the median and best class: nothing (against the best +0.91, worse)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Class x speed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Speed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Speed figures scaled by the class they were run in</t>
+  </si>
+  <si>
     <t xml:space="preserve">Not built</t>
   </si>
   <si>
-    <t xml:space="preserve">B4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Closing-sectional proxy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Speed over the final furlongs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not available</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No sectional or per-horse times in the data</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Headgear type flags</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Equipment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One flag per headgear item (blinkers, visor, cheekpieces, hood, tongue-tie)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Partial: one category column</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Age restriction</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Race conditions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Age band of the race (2yo, 3yo only, 3yo+, 4yo+)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">race_restrictions_age is never read</t>
-  </si>
-  <si>
-    <t xml:space="preserve">H3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Claimer flag</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Connections</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Whether the jockey claims an allowance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Partial: raw claim only; is_claimer is opt-in</t>
-  </si>
-  <si>
-    <t xml:space="preserve">I1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OR percentile in the field</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ratings</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Official rating's percentile within the race</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Partial: difference to the max and median only</t>
-  </si>
-  <si>
-    <t xml:space="preserve">I2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OR trajectory slope</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Slope of the official rating over recent runs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Partial: changes only</t>
-  </si>
-  <si>
-    <t xml:space="preserve">J1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Month / season</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Context</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Seasonal effects</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Surveyed on 24 Sep: nothing for the price to miss</t>
-  </si>
-  <si>
-    <t xml:space="preserve">J2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Day of week</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weekday effects (strength of meetings)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Surveyed: nothing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">J4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campaign stage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Run number within the current campaign</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Written in model/primitives.py, never called; fr_runs_since_break now covers most of it</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Major-race experience</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Class</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Runs and form in Group / Listed / major races</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Screened 27 Sep against the best model's errors (black-type runs, finishing position and win rate before today: +0.53 x 10^-4, nothing; research/queries/travel_residuals.py)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Class ladder vs career median</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Today's class against the horse's career median class</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Partial: against a three-run mean</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Class x speed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Speed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Speed figures scaled by the class they were run in</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weight per OR point</t>
+    <t xml:space="preserve">L5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weight against the last three runs</t>
   </si>
   <si>
     <t xml:space="preserve">Handicap</t>
   </si>
   <si>
-    <t xml:space="preserve">Weight carried relative to the official rating</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The handicap block's hc_wt_vs_mark is close (opt-in, added nothing against the result)</t>
+    <t xml:space="preserve">Weight carried today less the mean of its last three runs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Screened (research query misc_residuals, 27 Sep, x 10^-4 on the pair's mean |log error|): -2.14 (-3.64 to -0.62), resolved, the size of the handicap angles' read; the model reads the weight against the last run (weight_change_lr) only. The next small candidate for a fit</t>
   </si>
   <si>
     <t xml:space="preserve">R1</t>
@@ -10765,7 +10768,7 @@
       </c>
       <c r="B16" s="4" t="n">
         <f aca="false">COUNTIF('Not yet developed'!$G$2:$G$27,A16)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
@@ -10776,7 +10779,7 @@
       </c>
       <c r="B17" s="4" t="n">
         <f aca="false">COUNTIF('Not yet developed'!$G$2:$G$27,A17)</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
@@ -61943,7 +61946,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
         <v>3243</v>
       </c>
@@ -61963,7 +61966,7 @@
         <v>3246</v>
       </c>
       <c r="G3" s="13" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -61989,7 +61992,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
         <v>3252</v>
       </c>
@@ -62058,7 +62061,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
         <v>3267</v>
       </c>
@@ -62081,7 +62084,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
         <v>3272</v>
       </c>
@@ -62196,7 +62199,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
         <v>3294</v>
       </c>
@@ -62236,30 +62239,30 @@
         <v>3241</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>3246</v>
+        <v>3302</v>
       </c>
       <c r="G15" s="13" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>3302</v>
+        <v>3303</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>3303</v>
+        <v>3304</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>3304</v>
+        <v>3305</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>3305</v>
+        <v>3306</v>
       </c>
       <c r="E16" s="13" t="s">
         <v>3241</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>3306</v>
+        <v>3307</v>
       </c>
       <c r="G16" s="13" t="s">
         <v>14</v>
@@ -62267,22 +62270,22 @@
     </row>
     <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>3307</v>
+        <v>3308</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>3308</v>
+        <v>3309</v>
       </c>
       <c r="C17" s="13" t="s">
         <v>3264</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>3309</v>
+        <v>3310</v>
       </c>
       <c r="E17" s="13" t="s">
         <v>3241</v>
       </c>
       <c r="F17" s="13" t="s">
-        <v>3310</v>
+        <v>3311</v>
       </c>
       <c r="G17" s="13" t="s">
         <v>15</v>
@@ -62290,22 +62293,22 @@
     </row>
     <row r="18" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>3311</v>
+        <v>3312</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>3312</v>
+        <v>3313</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>3313</v>
+        <v>3314</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>3314</v>
+        <v>3315</v>
       </c>
       <c r="E18" s="13" t="s">
         <v>3241</v>
       </c>
       <c r="F18" s="13" t="s">
-        <v>3315</v>
+        <v>3316</v>
       </c>
       <c r="G18" s="13" t="s">
         <v>15</v>
@@ -62313,22 +62316,22 @@
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>3316</v>
+        <v>3317</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>3317</v>
+        <v>3318</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>3318</v>
+        <v>3319</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>3319</v>
+        <v>3320</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>3320</v>
+        <v>3321</v>
       </c>
       <c r="F19" s="13" t="s">
-        <v>3321</v>
+        <v>3322</v>
       </c>
       <c r="G19" s="13" t="s">
         <v>15</v>
@@ -62336,22 +62339,22 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>3322</v>
+        <v>3323</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>3323</v>
+        <v>3324</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>3324</v>
+        <v>3325</v>
       </c>
       <c r="D20" s="13" t="s">
-        <v>3325</v>
+        <v>3326</v>
       </c>
       <c r="E20" s="13" t="s">
         <v>3241</v>
       </c>
       <c r="F20" s="13" t="s">
-        <v>3326</v>
+        <v>3327</v>
       </c>
       <c r="G20" s="13" t="s">
         <v>14</v>
@@ -62359,22 +62362,22 @@
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="s">
-        <v>3327</v>
+        <v>3328</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>3328</v>
+        <v>3329</v>
       </c>
       <c r="C21" s="13" t="s">
         <v>3264</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>3329</v>
+        <v>3330</v>
       </c>
       <c r="E21" s="13" t="s">
         <v>3250</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>3330</v>
+        <v>3331</v>
       </c>
       <c r="G21" s="13" t="s">
         <v>16</v>
@@ -62382,22 +62385,22 @@
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>3331</v>
+        <v>3332</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>3332</v>
+        <v>3333</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>3333</v>
+        <v>3334</v>
       </c>
       <c r="D22" s="13" t="s">
-        <v>3334</v>
+        <v>3335</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>3335</v>
+        <v>3336</v>
       </c>
       <c r="F22" s="13" t="s">
-        <v>3336</v>
+        <v>3337</v>
       </c>
       <c r="G22" s="13" t="s">
         <v>15</v>
@@ -62405,22 +62408,22 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>3337</v>
+        <v>3338</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>3338</v>
+        <v>3339</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>3333</v>
+        <v>3334</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>3339</v>
+        <v>3340</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>3335</v>
+        <v>3336</v>
       </c>
       <c r="F23" s="13" t="s">
-        <v>3340</v>
+        <v>3341</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>15</v>
@@ -62428,22 +62431,22 @@
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>3341</v>
+        <v>3342</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>3342</v>
+        <v>3343</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>3333</v>
+        <v>3334</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>3343</v>
+        <v>3344</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>3335</v>
+        <v>3336</v>
       </c>
       <c r="F24" s="13" t="s">
-        <v>3344</v>
+        <v>3345</v>
       </c>
       <c r="G24" s="13" t="s">
         <v>15</v>
@@ -62451,22 +62454,22 @@
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>3345</v>
+        <v>3346</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>3346</v>
+        <v>3347</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>3333</v>
+        <v>3334</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>3347</v>
+        <v>3348</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>3335</v>
+        <v>3336</v>
       </c>
       <c r="F25" s="13" t="s">
-        <v>3348</v>
+        <v>3349</v>
       </c>
       <c r="G25" s="13" t="s">
         <v>14</v>
@@ -62474,22 +62477,22 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
-        <v>3349</v>
+        <v>3350</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>3350</v>
+        <v>3351</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>3333</v>
+        <v>3334</v>
       </c>
       <c r="D26" s="13" t="s">
-        <v>3351</v>
+        <v>3352</v>
       </c>
       <c r="E26" s="13" t="s">
-        <v>3335</v>
+        <v>3336</v>
       </c>
       <c r="F26" s="13" t="s">
-        <v>3352</v>
+        <v>3353</v>
       </c>
       <c r="G26" s="13" t="s">
         <v>15</v>
@@ -62497,22 +62500,22 @@
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
-        <v>3353</v>
+        <v>3354</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>3354</v>
+        <v>3355</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>3313</v>
+        <v>3314</v>
       </c>
       <c r="D27" s="13" t="s">
-        <v>3355</v>
+        <v>3356</v>
       </c>
       <c r="E27" s="13" t="s">
-        <v>3356</v>
+        <v>3357</v>
       </c>
       <c r="F27" s="13" t="s">
-        <v>3357</v>
+        <v>3358</v>
       </c>
       <c r="G27" s="13" t="s">
         <v>17</v>

</xml_diff>